<commit_message>
12 08 2025 12 27
</commit_message>
<xml_diff>
--- a/Книга1.xlsx
+++ b/Книга1.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9072" activeTab="4"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9072" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -17,6 +17,12 @@
     <sheet name="Лист4" sheetId="4" r:id="rId3"/>
     <sheet name="Лист5" sheetId="5" r:id="rId4"/>
     <sheet name="Лист6" sheetId="6" r:id="rId5"/>
+    <sheet name="Лист7" sheetId="7" r:id="rId6"/>
+    <sheet name="Лист8" sheetId="8" r:id="rId7"/>
+    <sheet name="Лист9" sheetId="9" r:id="rId8"/>
+    <sheet name="Лист10" sheetId="10" r:id="rId9"/>
+    <sheet name="Лист11" sheetId="11" r:id="rId10"/>
+    <sheet name="Лист12" sheetId="12" r:id="rId11"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -28,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="76">
   <si>
     <t>O’quv yillari</t>
   </si>
@@ -157,13 +163,179 @@
   </si>
   <si>
     <t>O‘zlashtirishi yuqori</t>
+  </si>
+  <si>
+    <t>3.2-jadval. Tajriba –sinov ishlarida ishtirok etgan oliy ta’lim muassasasi talabalari</t>
+  </si>
+  <si>
+    <t>3.3-jadval. Tajriba-sinov natijalari</t>
+  </si>
+  <si>
+    <t>3.4-jadval. Ikkinchi bosqich pedagogik tajriba-sinovlarning natijalari</t>
+  </si>
+  <si>
+    <t>3.5-jadval. Dastur ishlanmalarning ta’lim jarayoniga joriy qilinganligi nisbiy samaradorligi.</t>
+  </si>
+  <si>
+    <t>3.6-jadval. O‘zMU da olib borilgan tadqiqot natijalari.</t>
+  </si>
+  <si>
+    <t>O‘quv yili</t>
+  </si>
+  <si>
+    <t>Tajriba guruhi</t>
+  </si>
+  <si>
+    <t>Nazorat guruhi</t>
+  </si>
+  <si>
+    <t>Shakllanganlik darajasi</t>
+  </si>
+  <si>
+    <t>To‘liq</t>
+  </si>
+  <si>
+    <t>Asosan</t>
+  </si>
+  <si>
+    <t>Qisman</t>
+  </si>
+  <si>
+    <t>Past</t>
+  </si>
+  <si>
+    <t>2022-2023</t>
+  </si>
+  <si>
+    <t>3.7-jadval. TAFU da olib borilgan tadqiqot natijalari.</t>
+  </si>
+  <si>
+    <t>3.8-jadval. NamDPU da olib borilgan tadqiqot natijalari.</t>
+  </si>
+  <si>
+    <t>3.9-jadval.</t>
+  </si>
+  <si>
+    <t>Tanlanmalar</t>
+  </si>
+  <si>
+    <t>Nazorat gurhi</t>
+  </si>
+  <si>
+    <t>3.10-jadval.– jadval. Tajriba boshida tanlab olingan guruhlardagi o‘zlashtirish natijalari va gipoteza xulosasi.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tajriba </t>
+  </si>
+  <si>
+    <t>Nazorat</t>
+  </si>
+  <si>
+    <t>Tajriba.-sinov talabalar soni</t>
+  </si>
+  <si>
+    <t>Nazorat guruhi talabalr soni</t>
+  </si>
+  <si>
+    <r>
+      <t>X</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <vertAlign val="subscript"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+        <charset val="204"/>
+      </rPr>
+      <t>i</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="subscript"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+        <charset val="204"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+        <charset val="204"/>
+      </rPr>
+      <t>kvadrat</t>
+    </r>
+  </si>
+  <si>
+    <t>Kriteriya xulosasi</t>
+  </si>
+  <si>
+    <t>O‘zMU</t>
+  </si>
+  <si>
+    <r>
+      <t>H</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="subscript"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+        <charset val="204"/>
+      </rPr>
+      <t>0</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>H</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="subscript"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+        <charset val="204"/>
+      </rPr>
+      <t>1</t>
+    </r>
+  </si>
+  <si>
+    <t>3.11-jadval.– jadval. Tajriba boshida tanlab olingan guruhlardagi o‘zlashtirish natijalari va gipoteza xulosasi.</t>
+  </si>
+  <si>
+    <t>Tajriba</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.12-jadval. </t>
+  </si>
+  <si>
+    <t>Tajriba guruhidagi o‘rtacha o‘zlashtirish ko‘rsatkichi</t>
+  </si>
+  <si>
+    <t>Nazorat guruhidagi o‘rtacha o‘zlashtirish ko‘rsatkichi</t>
+  </si>
+  <si>
+    <t>Samaradorlik ko‘rsatkichlari</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -202,6 +374,47 @@
       <family val="1"/>
       <charset val="204"/>
     </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <i/>
+      <vertAlign val="subscript"/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <vertAlign val="subscript"/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <vertAlign val="subscript"/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="204"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -211,7 +424,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="22">
     <border>
       <left/>
       <right/>
@@ -328,11 +541,163 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thick">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thick">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -346,6 +711,46 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -361,21 +766,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
@@ -385,33 +775,141 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -552,7 +1050,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Лист5!$C$18</c:f>
+              <c:f>Лист5!$C$21</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -603,7 +1101,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Лист5!$B$19:$B$21</c:f>
+              <c:f>Лист5!$B$22:$B$24</c:f>
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
@@ -620,7 +1118,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Лист5!$C$19:$C$21</c:f>
+              <c:f>Лист5!$C$22:$C$24</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
@@ -647,7 +1145,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>Лист5!$E$18</c:f>
+              <c:f>Лист5!$E$21</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -698,7 +1196,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Лист5!$B$19:$B$21</c:f>
+              <c:f>Лист5!$B$22:$B$24</c:f>
               <c:strCache>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
@@ -715,7 +1213,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Лист5!$E$19:$E$21</c:f>
+              <c:f>Лист5!$E$22:$E$24</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
@@ -761,7 +1259,7 @@
                     <c:extLst>
                       <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                         <c15:formulaRef>
-                          <c15:sqref>Лист5!$D$18</c15:sqref>
+                          <c15:sqref>Лист5!$D$21</c15:sqref>
                         </c15:formulaRef>
                       </c:ext>
                     </c:extLst>
@@ -815,7 +1313,7 @@
                     <c:extLst>
                       <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                         <c15:formulaRef>
-                          <c15:sqref>Лист5!$B$19:$B$21</c15:sqref>
+                          <c15:sqref>Лист5!$B$22:$B$24</c15:sqref>
                         </c15:formulaRef>
                       </c:ext>
                     </c:extLst>
@@ -838,7 +1336,7 @@
                     <c:extLst>
                       <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                         <c15:formulaRef>
-                          <c15:sqref>Лист5!$D$19:$D$21</c15:sqref>
+                          <c15:sqref>Лист5!$D$22:$D$24</c15:sqref>
                         </c15:formulaRef>
                       </c:ext>
                     </c:extLst>
@@ -870,10 +1368,10 @@
                 <c:order val="3"/>
                 <c:tx>
                   <c:strRef>
-                    <c:extLst>
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
                       <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                         <c15:formulaRef>
-                          <c15:sqref>Лист5!$F$18</c15:sqref>
+                          <c15:sqref>Лист5!$F$21</c15:sqref>
                         </c15:formulaRef>
                       </c:ext>
                     </c:extLst>
@@ -927,10 +1425,10 @@
                 <c:invertIfNegative val="0"/>
                 <c:cat>
                   <c:strRef>
-                    <c:extLst>
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
                       <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                         <c15:formulaRef>
-                          <c15:sqref>Лист5!$B$19:$B$21</c15:sqref>
+                          <c15:sqref>Лист5!$B$22:$B$24</c15:sqref>
                         </c15:formulaRef>
                       </c:ext>
                     </c:extLst>
@@ -950,10 +1448,10 @@
                 </c:cat>
                 <c:val>
                   <c:numRef>
-                    <c:extLst>
+                    <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
                       <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                         <c15:formulaRef>
-                          <c15:sqref>Лист5!$F$19:$F$21</c15:sqref>
+                          <c15:sqref>Лист5!$F$22:$F$24</c15:sqref>
                         </c15:formulaRef>
                       </c:ext>
                     </c:extLst>
@@ -972,7 +1470,7 @@
                     </c:numCache>
                   </c:numRef>
                 </c:val>
-                <c:extLst>
+                <c:extLst xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
                   <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                     <c16:uniqueId val="{00000003-A364-4E5C-9039-6E34970B2DF4}"/>
                   </c:ext>
@@ -1713,14 +2211,14 @@
         <xdr:from>
           <xdr:col>1</xdr:col>
           <xdr:colOff>0</xdr:colOff>
-          <xdr:row>2</xdr:row>
+          <xdr:row>5</xdr:row>
           <xdr:rowOff>0</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>2</xdr:col>
           <xdr:colOff>0</xdr:colOff>
-          <xdr:row>2</xdr:row>
-          <xdr:rowOff>613410</xdr:rowOff>
+          <xdr:row>5</xdr:row>
+          <xdr:rowOff>617220</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -1764,14 +2262,14 @@
         <xdr:from>
           <xdr:col>2</xdr:col>
           <xdr:colOff>106680</xdr:colOff>
-          <xdr:row>2</xdr:row>
+          <xdr:row>5</xdr:row>
           <xdr:rowOff>53340</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>2</xdr:col>
           <xdr:colOff>1074420</xdr:colOff>
-          <xdr:row>2</xdr:row>
-          <xdr:rowOff>730879</xdr:rowOff>
+          <xdr:row>5</xdr:row>
+          <xdr:rowOff>731520</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -1815,14 +2313,14 @@
         <xdr:from>
           <xdr:col>3</xdr:col>
           <xdr:colOff>0</xdr:colOff>
-          <xdr:row>2</xdr:row>
-          <xdr:rowOff>1</xdr:rowOff>
+          <xdr:row>5</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>3</xdr:col>
           <xdr:colOff>1135380</xdr:colOff>
-          <xdr:row>2</xdr:row>
-          <xdr:rowOff>673971</xdr:rowOff>
+          <xdr:row>5</xdr:row>
+          <xdr:rowOff>670560</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -1866,14 +2364,14 @@
         <xdr:from>
           <xdr:col>4</xdr:col>
           <xdr:colOff>0</xdr:colOff>
-          <xdr:row>2</xdr:row>
+          <xdr:row>5</xdr:row>
           <xdr:rowOff>0</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>4</xdr:col>
           <xdr:colOff>944880</xdr:colOff>
-          <xdr:row>2</xdr:row>
-          <xdr:rowOff>732183</xdr:rowOff>
+          <xdr:row>5</xdr:row>
+          <xdr:rowOff>731520</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -1917,14 +2415,14 @@
         <xdr:from>
           <xdr:col>5</xdr:col>
           <xdr:colOff>0</xdr:colOff>
-          <xdr:row>2</xdr:row>
+          <xdr:row>5</xdr:row>
           <xdr:rowOff>0</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>5</xdr:col>
           <xdr:colOff>1013460</xdr:colOff>
-          <xdr:row>2</xdr:row>
-          <xdr:rowOff>676780</xdr:rowOff>
+          <xdr:row>5</xdr:row>
+          <xdr:rowOff>678180</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -1968,14 +2466,14 @@
         <xdr:from>
           <xdr:col>6</xdr:col>
           <xdr:colOff>0</xdr:colOff>
-          <xdr:row>2</xdr:row>
+          <xdr:row>5</xdr:row>
           <xdr:rowOff>0</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>6</xdr:col>
           <xdr:colOff>868680</xdr:colOff>
-          <xdr:row>2</xdr:row>
-          <xdr:rowOff>752696</xdr:rowOff>
+          <xdr:row>5</xdr:row>
+          <xdr:rowOff>754380</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -2017,13 +2515,13 @@
     <xdr:from>
       <xdr:col>8</xdr:col>
       <xdr:colOff>87085</xdr:colOff>
-      <xdr:row>4</xdr:row>
+      <xdr:row>7</xdr:row>
       <xdr:rowOff>484414</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>15</xdr:col>
       <xdr:colOff>391885</xdr:colOff>
-      <xdr:row>12</xdr:row>
+      <xdr:row>15</xdr:row>
       <xdr:rowOff>375557</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -2043,6 +2541,725 @@
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor>
+        <xdr:from>
+          <xdr:col>3</xdr:col>
+          <xdr:colOff>0</xdr:colOff>
+          <xdr:row>3</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>3</xdr:col>
+          <xdr:colOff>487680</xdr:colOff>
+          <xdr:row>3</xdr:row>
+          <xdr:rowOff>220980</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="11278" name="Object 14" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s11278"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:extLst>
+              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+                <a14:hiddenFill>
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF"/>
+                  </a:solidFill>
+                </a14:hiddenFill>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+        </xdr:sp>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor>
+        <xdr:from>
+          <xdr:col>4</xdr:col>
+          <xdr:colOff>0</xdr:colOff>
+          <xdr:row>3</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>4</xdr:col>
+          <xdr:colOff>487680</xdr:colOff>
+          <xdr:row>3</xdr:row>
+          <xdr:rowOff>220980</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="11277" name="Object 13" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s11277"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:extLst>
+              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+                <a14:hiddenFill>
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF"/>
+                  </a:solidFill>
+                </a14:hiddenFill>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+        </xdr:sp>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor>
+        <xdr:from>
+          <xdr:col>5</xdr:col>
+          <xdr:colOff>0</xdr:colOff>
+          <xdr:row>3</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>5</xdr:col>
+          <xdr:colOff>541020</xdr:colOff>
+          <xdr:row>3</xdr:row>
+          <xdr:rowOff>228600</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="11276" name="Object 12" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s11276"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:extLst>
+              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+                <a14:hiddenFill>
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF"/>
+                  </a:solidFill>
+                </a14:hiddenFill>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+        </xdr:sp>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor>
+        <xdr:from>
+          <xdr:col>6</xdr:col>
+          <xdr:colOff>0</xdr:colOff>
+          <xdr:row>3</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>6</xdr:col>
+          <xdr:colOff>495300</xdr:colOff>
+          <xdr:row>3</xdr:row>
+          <xdr:rowOff>220980</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="11275" name="Object 11" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s11275"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:extLst>
+              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+                <a14:hiddenFill>
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF"/>
+                  </a:solidFill>
+                </a14:hiddenFill>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+        </xdr:sp>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor>
+        <xdr:from>
+          <xdr:col>7</xdr:col>
+          <xdr:colOff>0</xdr:colOff>
+          <xdr:row>3</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>7</xdr:col>
+          <xdr:colOff>480060</xdr:colOff>
+          <xdr:row>3</xdr:row>
+          <xdr:rowOff>220980</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="11274" name="Object 10" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s11274"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:extLst>
+              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+                <a14:hiddenFill>
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF"/>
+                  </a:solidFill>
+                </a14:hiddenFill>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+        </xdr:sp>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor>
+        <xdr:from>
+          <xdr:col>3</xdr:col>
+          <xdr:colOff>0</xdr:colOff>
+          <xdr:row>4</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>3</xdr:col>
+          <xdr:colOff>480060</xdr:colOff>
+          <xdr:row>4</xdr:row>
+          <xdr:rowOff>220980</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="11273" name="Object 9" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s11273"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:extLst>
+              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+                <a14:hiddenFill>
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF"/>
+                  </a:solidFill>
+                </a14:hiddenFill>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+        </xdr:sp>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor>
+        <xdr:from>
+          <xdr:col>4</xdr:col>
+          <xdr:colOff>0</xdr:colOff>
+          <xdr:row>4</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>4</xdr:col>
+          <xdr:colOff>502920</xdr:colOff>
+          <xdr:row>4</xdr:row>
+          <xdr:rowOff>220980</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="11272" name="Object 8" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s11272"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:extLst>
+              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+                <a14:hiddenFill>
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF"/>
+                  </a:solidFill>
+                </a14:hiddenFill>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+        </xdr:sp>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor>
+        <xdr:from>
+          <xdr:col>5</xdr:col>
+          <xdr:colOff>0</xdr:colOff>
+          <xdr:row>4</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>5</xdr:col>
+          <xdr:colOff>563880</xdr:colOff>
+          <xdr:row>4</xdr:row>
+          <xdr:rowOff>228600</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="11271" name="Object 7" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s11271"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:extLst>
+              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+                <a14:hiddenFill>
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF"/>
+                  </a:solidFill>
+                </a14:hiddenFill>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+        </xdr:sp>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor>
+        <xdr:from>
+          <xdr:col>6</xdr:col>
+          <xdr:colOff>0</xdr:colOff>
+          <xdr:row>4</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>6</xdr:col>
+          <xdr:colOff>563880</xdr:colOff>
+          <xdr:row>4</xdr:row>
+          <xdr:rowOff>220980</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="11270" name="Object 6" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s11270"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:extLst>
+              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+                <a14:hiddenFill>
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF"/>
+                  </a:solidFill>
+                </a14:hiddenFill>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+        </xdr:sp>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor>
+        <xdr:from>
+          <xdr:col>7</xdr:col>
+          <xdr:colOff>0</xdr:colOff>
+          <xdr:row>4</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>7</xdr:col>
+          <xdr:colOff>487680</xdr:colOff>
+          <xdr:row>4</xdr:row>
+          <xdr:rowOff>220980</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="11269" name="Object 5" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s11269"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:extLst>
+              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+                <a14:hiddenFill>
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF"/>
+                  </a:solidFill>
+                </a14:hiddenFill>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+        </xdr:sp>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor>
+        <xdr:from>
+          <xdr:col>3</xdr:col>
+          <xdr:colOff>0</xdr:colOff>
+          <xdr:row>5</xdr:row>
+          <xdr:rowOff>30760</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>3</xdr:col>
+          <xdr:colOff>1196340</xdr:colOff>
+          <xdr:row>5</xdr:row>
+          <xdr:rowOff>213359</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="11268" name="Object 4" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s11268"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:extLst>
+              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+                <a14:hiddenFill>
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF"/>
+                  </a:solidFill>
+                </a14:hiddenFill>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+        </xdr:sp>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor>
+        <xdr:from>
+          <xdr:col>4</xdr:col>
+          <xdr:colOff>0</xdr:colOff>
+          <xdr:row>5</xdr:row>
+          <xdr:rowOff>49862</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>4</xdr:col>
+          <xdr:colOff>1150620</xdr:colOff>
+          <xdr:row>5</xdr:row>
+          <xdr:rowOff>220980</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="11267" name="Object 3" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s11267"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:extLst>
+              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+                <a14:hiddenFill>
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF"/>
+                  </a:solidFill>
+                </a14:hiddenFill>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+        </xdr:sp>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor>
+        <xdr:from>
+          <xdr:col>5</xdr:col>
+          <xdr:colOff>0</xdr:colOff>
+          <xdr:row>5</xdr:row>
+          <xdr:rowOff>53108</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>5</xdr:col>
+          <xdr:colOff>1158240</xdr:colOff>
+          <xdr:row>5</xdr:row>
+          <xdr:rowOff>228599</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="11266" name="Object 2" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s11266"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:extLst>
+              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+                <a14:hiddenFill>
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF"/>
+                  </a:solidFill>
+                </a14:hiddenFill>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+        </xdr:sp>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor>
+        <xdr:from>
+          <xdr:col>6</xdr:col>
+          <xdr:colOff>0</xdr:colOff>
+          <xdr:row>5</xdr:row>
+          <xdr:rowOff>46300</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>6</xdr:col>
+          <xdr:colOff>1264920</xdr:colOff>
+          <xdr:row>5</xdr:row>
+          <xdr:rowOff>220979</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="11265" name="Object 1" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s11265"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:extLst>
+              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+                <a14:hiddenFill>
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF"/>
+                  </a:solidFill>
+                </a14:hiddenFill>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+        </xdr:sp>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
 </xdr:wsDr>
 </file>
 
@@ -2309,7 +3526,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B3:E15"/>
+  <dimension ref="B2:E15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="20.33203125" customWidth="1"/>
@@ -2317,21 +3534,29 @@
     <col min="5" max="5" width="19.6640625" customWidth="1"/>
   </cols>
   <sheetData>
+    <row r="2" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B2" s="30" t="s">
+        <v>41</v>
+      </c>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+    </row>
     <row r="3" spans="2:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="4" spans="2:5" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="8"/>
+      <c r="D4" s="22"/>
       <c r="E4" s="1" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="5" spans="2:5" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="6"/>
+      <c r="B5" s="20"/>
       <c r="C5" s="2" t="s">
         <v>3</v>
       </c>
@@ -2343,12 +3568,12 @@
       </c>
     </row>
     <row r="6" spans="2:5" ht="42.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="9"/>
-      <c r="D6" s="9"/>
-      <c r="E6" s="8"/>
+      <c r="C6" s="23"/>
+      <c r="D6" s="23"/>
+      <c r="E6" s="22"/>
     </row>
     <row r="7" spans="2:5" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B7" s="3" t="s">
@@ -2381,12 +3606,12 @@
       </c>
     </row>
     <row r="9" spans="2:5" ht="48" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="9"/>
-      <c r="D9" s="9"/>
-      <c r="E9" s="8"/>
+      <c r="C9" s="23"/>
+      <c r="D9" s="23"/>
+      <c r="E9" s="22"/>
     </row>
     <row r="10" spans="2:5" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B10" s="3" t="s">
@@ -2419,12 +3644,12 @@
       </c>
     </row>
     <row r="12" spans="2:5" ht="34.200000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="C12" s="9"/>
-      <c r="D12" s="9"/>
-      <c r="E12" s="8"/>
+      <c r="C12" s="23"/>
+      <c r="D12" s="23"/>
+      <c r="E12" s="22"/>
     </row>
     <row r="13" spans="2:5" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B13" s="3" t="s">
@@ -2474,7 +3699,8 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
+    <mergeCell ref="B2:E2"/>
     <mergeCell ref="B4:B5"/>
     <mergeCell ref="C4:D4"/>
     <mergeCell ref="B6:E6"/>
@@ -2486,9 +3712,593 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="D3:P15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="3" spans="4:16" ht="18" x14ac:dyDescent="0.3">
+      <c r="D3" s="69" t="s">
+        <v>70</v>
+      </c>
+      <c r="E3" s="69"/>
+      <c r="F3" s="69"/>
+      <c r="G3" s="69"/>
+      <c r="H3" s="69"/>
+      <c r="I3" s="69"/>
+      <c r="J3" s="69"/>
+      <c r="K3" s="69"/>
+    </row>
+    <row r="4" spans="4:16" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="5" spans="4:16" ht="32.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D5" s="57" t="s">
+        <v>46</v>
+      </c>
+      <c r="E5" s="59" t="s">
+        <v>71</v>
+      </c>
+      <c r="F5" s="23"/>
+      <c r="G5" s="23"/>
+      <c r="H5" s="60"/>
+      <c r="I5" s="61" t="s">
+        <v>62</v>
+      </c>
+      <c r="J5" s="36"/>
+      <c r="K5" s="36"/>
+      <c r="L5" s="62"/>
+      <c r="M5" s="63" t="s">
+        <v>63</v>
+      </c>
+      <c r="N5" s="65" t="s">
+        <v>64</v>
+      </c>
+      <c r="O5" s="67" t="s">
+        <v>65</v>
+      </c>
+      <c r="P5" s="67" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="6" spans="4:16" ht="67.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D6" s="58"/>
+      <c r="E6" s="32" t="s">
+        <v>50</v>
+      </c>
+      <c r="F6" s="32" t="s">
+        <v>51</v>
+      </c>
+      <c r="G6" s="32" t="s">
+        <v>52</v>
+      </c>
+      <c r="H6" s="54" t="s">
+        <v>53</v>
+      </c>
+      <c r="I6" s="32" t="s">
+        <v>50</v>
+      </c>
+      <c r="J6" s="32" t="s">
+        <v>51</v>
+      </c>
+      <c r="K6" s="32" t="s">
+        <v>52</v>
+      </c>
+      <c r="L6" s="54" t="s">
+        <v>53</v>
+      </c>
+      <c r="M6" s="64"/>
+      <c r="N6" s="66"/>
+      <c r="O6" s="68"/>
+      <c r="P6" s="68"/>
+    </row>
+    <row r="7" spans="4:16" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D7" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="E7" s="23"/>
+      <c r="F7" s="23"/>
+      <c r="G7" s="23"/>
+      <c r="H7" s="23"/>
+      <c r="I7" s="23"/>
+      <c r="J7" s="23"/>
+      <c r="K7" s="23"/>
+      <c r="L7" s="23"/>
+      <c r="M7" s="23"/>
+      <c r="N7" s="23"/>
+      <c r="O7" s="23"/>
+      <c r="P7" s="22"/>
+    </row>
+    <row r="8" spans="4:16" ht="35.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D8" s="70" t="s">
+        <v>54</v>
+      </c>
+      <c r="E8" s="2">
+        <v>2</v>
+      </c>
+      <c r="F8" s="2">
+        <v>8</v>
+      </c>
+      <c r="G8" s="2">
+        <v>10</v>
+      </c>
+      <c r="H8" s="71">
+        <v>6</v>
+      </c>
+      <c r="I8" s="2">
+        <v>1</v>
+      </c>
+      <c r="J8" s="2">
+        <v>7</v>
+      </c>
+      <c r="K8" s="2">
+        <v>10</v>
+      </c>
+      <c r="L8" s="71">
+        <v>10</v>
+      </c>
+      <c r="M8" s="2">
+        <v>26</v>
+      </c>
+      <c r="N8" s="2">
+        <v>28</v>
+      </c>
+      <c r="O8" s="2">
+        <v>1.33</v>
+      </c>
+      <c r="P8" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="9" spans="4:16" ht="35.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D9" s="70" t="s">
+        <v>8</v>
+      </c>
+      <c r="E9" s="2">
+        <v>2</v>
+      </c>
+      <c r="F9" s="2">
+        <v>7</v>
+      </c>
+      <c r="G9" s="2">
+        <v>8</v>
+      </c>
+      <c r="H9" s="71">
+        <v>8</v>
+      </c>
+      <c r="I9" s="2">
+        <v>2</v>
+      </c>
+      <c r="J9" s="2">
+        <v>5</v>
+      </c>
+      <c r="K9" s="2">
+        <v>10</v>
+      </c>
+      <c r="L9" s="71">
+        <v>9</v>
+      </c>
+      <c r="M9" s="2">
+        <v>25</v>
+      </c>
+      <c r="N9" s="2">
+        <v>26</v>
+      </c>
+      <c r="O9" s="2">
+        <v>0.6</v>
+      </c>
+      <c r="P9" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="10" spans="4:16" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D10" s="21" t="s">
+        <v>9</v>
+      </c>
+      <c r="E10" s="23"/>
+      <c r="F10" s="23"/>
+      <c r="G10" s="23"/>
+      <c r="H10" s="23"/>
+      <c r="I10" s="23"/>
+      <c r="J10" s="23"/>
+      <c r="K10" s="23"/>
+      <c r="L10" s="23"/>
+      <c r="M10" s="23"/>
+      <c r="N10" s="23"/>
+      <c r="O10" s="23"/>
+      <c r="P10" s="22"/>
+    </row>
+    <row r="11" spans="4:16" ht="35.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D11" s="70" t="s">
+        <v>54</v>
+      </c>
+      <c r="E11" s="2">
+        <v>2</v>
+      </c>
+      <c r="F11" s="2">
+        <v>8</v>
+      </c>
+      <c r="G11" s="2">
+        <v>10</v>
+      </c>
+      <c r="H11" s="71">
+        <v>6</v>
+      </c>
+      <c r="I11" s="2">
+        <v>1</v>
+      </c>
+      <c r="J11" s="2">
+        <v>7</v>
+      </c>
+      <c r="K11" s="2">
+        <v>10</v>
+      </c>
+      <c r="L11" s="71">
+        <v>10</v>
+      </c>
+      <c r="M11" s="2">
+        <v>26</v>
+      </c>
+      <c r="N11" s="2">
+        <v>28</v>
+      </c>
+      <c r="O11" s="2">
+        <v>1.33</v>
+      </c>
+      <c r="P11" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="12" spans="4:16" ht="35.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D12" s="70" t="s">
+        <v>8</v>
+      </c>
+      <c r="E12" s="2">
+        <v>2</v>
+      </c>
+      <c r="F12" s="2">
+        <v>7</v>
+      </c>
+      <c r="G12" s="2">
+        <v>8</v>
+      </c>
+      <c r="H12" s="71">
+        <v>8</v>
+      </c>
+      <c r="I12" s="2">
+        <v>2</v>
+      </c>
+      <c r="J12" s="2">
+        <v>5</v>
+      </c>
+      <c r="K12" s="2">
+        <v>10</v>
+      </c>
+      <c r="L12" s="71">
+        <v>9</v>
+      </c>
+      <c r="M12" s="2">
+        <v>25</v>
+      </c>
+      <c r="N12" s="2">
+        <v>26</v>
+      </c>
+      <c r="O12" s="2">
+        <v>0.6</v>
+      </c>
+      <c r="P12" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="13" spans="4:16" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D13" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="E13" s="23"/>
+      <c r="F13" s="23"/>
+      <c r="G13" s="23"/>
+      <c r="H13" s="23"/>
+      <c r="I13" s="23"/>
+      <c r="J13" s="23"/>
+      <c r="K13" s="23"/>
+      <c r="L13" s="23"/>
+      <c r="M13" s="23"/>
+      <c r="N13" s="23"/>
+      <c r="O13" s="23"/>
+      <c r="P13" s="22"/>
+    </row>
+    <row r="14" spans="4:16" ht="35.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D14" s="70" t="s">
+        <v>54</v>
+      </c>
+      <c r="E14" s="2">
+        <v>2</v>
+      </c>
+      <c r="F14" s="2">
+        <v>8</v>
+      </c>
+      <c r="G14" s="2">
+        <v>10</v>
+      </c>
+      <c r="H14" s="71">
+        <v>6</v>
+      </c>
+      <c r="I14" s="2">
+        <v>1</v>
+      </c>
+      <c r="J14" s="2">
+        <v>7</v>
+      </c>
+      <c r="K14" s="2">
+        <v>10</v>
+      </c>
+      <c r="L14" s="71">
+        <v>10</v>
+      </c>
+      <c r="M14" s="2">
+        <v>26</v>
+      </c>
+      <c r="N14" s="2">
+        <v>28</v>
+      </c>
+      <c r="O14" s="2">
+        <v>1.33</v>
+      </c>
+      <c r="P14" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="15" spans="4:16" ht="35.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D15" s="70" t="s">
+        <v>8</v>
+      </c>
+      <c r="E15" s="2">
+        <v>2</v>
+      </c>
+      <c r="F15" s="2">
+        <v>7</v>
+      </c>
+      <c r="G15" s="2">
+        <v>8</v>
+      </c>
+      <c r="H15" s="71">
+        <v>8</v>
+      </c>
+      <c r="I15" s="2">
+        <v>2</v>
+      </c>
+      <c r="J15" s="2">
+        <v>5</v>
+      </c>
+      <c r="K15" s="2">
+        <v>10</v>
+      </c>
+      <c r="L15" s="71">
+        <v>9</v>
+      </c>
+      <c r="M15" s="2">
+        <v>25</v>
+      </c>
+      <c r="N15" s="2">
+        <v>26</v>
+      </c>
+      <c r="O15" s="2">
+        <v>0.6</v>
+      </c>
+      <c r="P15" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="11">
+    <mergeCell ref="O5:O6"/>
+    <mergeCell ref="P5:P6"/>
+    <mergeCell ref="D7:P7"/>
+    <mergeCell ref="D10:P10"/>
+    <mergeCell ref="D13:P13"/>
+    <mergeCell ref="D3:K3"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:H5"/>
+    <mergeCell ref="I5:L5"/>
+    <mergeCell ref="M5:M6"/>
+    <mergeCell ref="N5:N6"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="D2:G16"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="4" max="4" width="13.44140625" customWidth="1"/>
+    <col min="5" max="5" width="18.77734375" customWidth="1"/>
+    <col min="6" max="6" width="17.6640625" customWidth="1"/>
+    <col min="7" max="7" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="4:7" ht="36" x14ac:dyDescent="0.3">
+      <c r="D2" s="39" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="3" spans="4:7" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="4" spans="4:7" ht="162.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D4" s="72" t="s">
+        <v>46</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="5" spans="4:7" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D5" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="E5" s="23"/>
+      <c r="F5" s="23"/>
+      <c r="G5" s="22"/>
+    </row>
+    <row r="6" spans="4:7" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D6" s="40" t="s">
+        <v>54</v>
+      </c>
+      <c r="E6" s="2">
+        <v>76.11</v>
+      </c>
+      <c r="F6" s="2">
+        <v>67.14</v>
+      </c>
+      <c r="G6" s="2">
+        <v>1.1299999999999999</v>
+      </c>
+    </row>
+    <row r="7" spans="4:7" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D7" s="40" t="s">
+        <v>7</v>
+      </c>
+      <c r="E7" s="2">
+        <v>74.64</v>
+      </c>
+      <c r="F7" s="2">
+        <v>65.42</v>
+      </c>
+      <c r="G7" s="2">
+        <v>1.1399999999999999</v>
+      </c>
+    </row>
+    <row r="8" spans="4:7" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D8" s="40" t="s">
+        <v>8</v>
+      </c>
+      <c r="E8" s="2">
+        <v>75.39</v>
+      </c>
+      <c r="F8" s="2">
+        <v>66.31</v>
+      </c>
+      <c r="G8" s="2">
+        <v>1.1399999999999999</v>
+      </c>
+    </row>
+    <row r="9" spans="4:7" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D9" s="21" t="s">
+        <v>9</v>
+      </c>
+      <c r="E9" s="23"/>
+      <c r="F9" s="23"/>
+      <c r="G9" s="22"/>
+    </row>
+    <row r="10" spans="4:7" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D10" s="40" t="s">
+        <v>54</v>
+      </c>
+      <c r="E10" s="2">
+        <v>76.11</v>
+      </c>
+      <c r="F10" s="2">
+        <v>67.14</v>
+      </c>
+      <c r="G10" s="2">
+        <v>1.1299999999999999</v>
+      </c>
+    </row>
+    <row r="11" spans="4:7" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D11" s="40" t="s">
+        <v>7</v>
+      </c>
+      <c r="E11" s="2">
+        <v>74.64</v>
+      </c>
+      <c r="F11" s="2">
+        <v>65.42</v>
+      </c>
+      <c r="G11" s="2">
+        <v>1.1399999999999999</v>
+      </c>
+    </row>
+    <row r="12" spans="4:7" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D12" s="40" t="s">
+        <v>8</v>
+      </c>
+      <c r="E12" s="2">
+        <v>75.39</v>
+      </c>
+      <c r="F12" s="2">
+        <v>66.31</v>
+      </c>
+      <c r="G12" s="2">
+        <v>1.1399999999999999</v>
+      </c>
+    </row>
+    <row r="13" spans="4:7" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D13" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="E13" s="23"/>
+      <c r="F13" s="23"/>
+      <c r="G13" s="22"/>
+    </row>
+    <row r="14" spans="4:7" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D14" s="40" t="s">
+        <v>54</v>
+      </c>
+      <c r="E14" s="2">
+        <v>76.11</v>
+      </c>
+      <c r="F14" s="2">
+        <v>67.14</v>
+      </c>
+      <c r="G14" s="2">
+        <v>1.1299999999999999</v>
+      </c>
+    </row>
+    <row r="15" spans="4:7" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D15" s="40" t="s">
+        <v>7</v>
+      </c>
+      <c r="E15" s="2">
+        <v>74.64</v>
+      </c>
+      <c r="F15" s="2">
+        <v>65.42</v>
+      </c>
+      <c r="G15" s="2">
+        <v>1.1399999999999999</v>
+      </c>
+    </row>
+    <row r="16" spans="4:7" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D16" s="40" t="s">
+        <v>8</v>
+      </c>
+      <c r="E16" s="2">
+        <v>75.39</v>
+      </c>
+      <c r="F16" s="2">
+        <v>66.31</v>
+      </c>
+      <c r="G16" s="2">
+        <v>1.1399999999999999</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="D5:G5"/>
+    <mergeCell ref="D9:G9"/>
+    <mergeCell ref="D13:G13"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A2:E8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.88671875" customWidth="1"/>
@@ -2498,72 +4308,81 @@
     <col min="5" max="5" width="23.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="72" x14ac:dyDescent="0.3">
-      <c r="A1" s="10" t="s">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C2" s="30" t="s">
+        <v>42</v>
+      </c>
+      <c r="D2" s="30"/>
+    </row>
+    <row r="4" spans="1:5" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B4" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C4" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D4" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E4" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="18" x14ac:dyDescent="0.3">
-      <c r="A2" s="10">
+    <row r="5" spans="1:5" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="7">
         <v>1</v>
       </c>
-      <c r="B2" s="10" t="s">
+      <c r="B5" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="10">
-        <v>5.21</v>
-      </c>
-      <c r="D2" s="10">
-        <v>4.6500000000000004</v>
-      </c>
-      <c r="E2" s="10">
-        <v>88.2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="18" x14ac:dyDescent="0.3">
-      <c r="A3" s="10">
+      <c r="C5" s="72">
+        <v>4.91</v>
+      </c>
+      <c r="D5" s="6">
+        <v>3.37</v>
+      </c>
+      <c r="E5" s="6">
+        <v>68.599999999999994</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="7">
         <v>2</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B6" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="10">
-        <v>8.33</v>
-      </c>
-      <c r="D3" s="10">
-        <v>4.0599999999999996</v>
-      </c>
-      <c r="E3" s="10">
-        <v>42.5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="C5" s="11">
-        <f>C3/C2</f>
-        <v>1.5988483685220729</v>
-      </c>
-      <c r="D5" s="11">
-        <f t="shared" ref="D5:E5" si="0">D3/D2</f>
-        <v>0.8731182795698923</v>
-      </c>
-      <c r="E5" s="11">
+      <c r="C6" s="5">
+        <v>7.98</v>
+      </c>
+      <c r="D6" s="2">
+        <v>2.4500000000000002</v>
+      </c>
+      <c r="E6" s="2">
+        <v>30.7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C8" s="8">
+        <f>C6/C5</f>
+        <v>1.6252545824847251</v>
+      </c>
+      <c r="D8" s="8">
+        <f t="shared" ref="D8:E8" si="0">D6/D5</f>
+        <v>0.72700296735905046</v>
+      </c>
+      <c r="E8" s="8">
         <f t="shared" si="0"/>
-        <v>0.48185941043083896</v>
+        <v>0.44752186588921283</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="C2:D2"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
@@ -2571,179 +4390,185 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H7"/>
+  <dimension ref="A2:H10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:8" ht="42" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="15" t="s">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="D2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="4" spans="1:8" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B4" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C4" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="D1" s="9"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="7" t="s">
+      <c r="D4" s="23"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="G1" s="9"/>
-      <c r="H1" s="8"/>
-    </row>
-    <row r="2" spans="1:8" ht="93.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="16"/>
-      <c r="B2" s="5"/>
-      <c r="C2" s="13" t="s">
+      <c r="G4" s="23"/>
+      <c r="H4" s="22"/>
+    </row>
+    <row r="5" spans="1:8" ht="93.6" x14ac:dyDescent="0.3">
+      <c r="A5" s="25"/>
+      <c r="B5" s="19"/>
+      <c r="C5" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="D5" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="E5" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="F2" s="13" t="s">
+      <c r="F5" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="G2" s="13" t="s">
+      <c r="G5" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="H2" s="13" t="s">
+      <c r="H5" s="10" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="16.8" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="17"/>
-      <c r="B3" s="6"/>
-      <c r="C3" s="14" t="s">
+    <row r="6" spans="1:8" ht="16.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="26"/>
+      <c r="B6" s="20"/>
+      <c r="C6" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="D3" s="14" t="s">
+      <c r="D6" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="E3" s="14" t="s">
+      <c r="E6" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="F3" s="14" t="s">
+      <c r="F6" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="G3" s="14" t="s">
+      <c r="G6" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="H3" s="14" t="s">
+      <c r="H6" s="11" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="71.400000000000006" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="15" t="s">
+    <row r="7" spans="1:8" ht="71.400000000000006" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="24" t="s">
         <v>29</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B7" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C7" s="2">
         <v>5.5</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D7" s="2">
         <v>2.9</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E7" s="2">
         <v>0.89</v>
       </c>
-      <c r="F4" s="2">
+      <c r="F7" s="2">
         <v>6</v>
       </c>
-      <c r="G4" s="2">
+      <c r="G7" s="2">
         <v>2.54</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H7" s="2">
         <v>0.89</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="17"/>
-      <c r="B5" s="2" t="s">
+    <row r="8" spans="1:8" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="26"/>
+      <c r="B8" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C5" s="2">
+      <c r="C8" s="2">
         <v>7.3</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D8" s="2">
         <v>2.5</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E8" s="2">
         <v>0.75</v>
       </c>
-      <c r="F5" s="2">
+      <c r="F8" s="2">
         <v>8</v>
       </c>
-      <c r="G5" s="2">
+      <c r="G8" s="2">
         <v>2.27</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H8" s="2">
         <v>0.71</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="71.400000000000006" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="15" t="s">
+    <row r="9" spans="1:8" ht="71.400000000000006" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="24" t="s">
         <v>32</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B9" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C6" s="2">
+      <c r="C9" s="2">
         <v>6.4</v>
       </c>
-      <c r="D6" s="2">
+      <c r="D9" s="2">
         <v>2.78</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E9" s="2">
         <v>0.91</v>
       </c>
-      <c r="F6" s="2">
+      <c r="F9" s="2">
         <v>6.6</v>
       </c>
-      <c r="G6" s="2">
+      <c r="G9" s="2">
         <v>2.31</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H9" s="2">
         <v>0.76</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="17"/>
-      <c r="B7" s="2" t="s">
+    <row r="10" spans="1:8" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="26"/>
+      <c r="B10" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C7" s="2">
+      <c r="C10" s="2">
         <v>8.1999999999999993</v>
       </c>
-      <c r="D7" s="2">
+      <c r="D10" s="2">
         <v>1.78</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E10" s="2">
         <v>0.56999999999999995</v>
       </c>
-      <c r="F7" s="2">
+      <c r="F10" s="2">
         <v>8.6</v>
       </c>
-      <c r="G7" s="2">
+      <c r="G10" s="2">
         <v>1.69</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H10" s="2">
         <v>0.56000000000000005</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A1:A3"/>
-    <mergeCell ref="C1:E1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="A4:A5"/>
-    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="A4:A6"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="F4:H4"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="A7:A8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2751,7 +4576,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G36"/>
+  <dimension ref="A2:G39"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.5546875" customWidth="1"/>
@@ -2763,287 +4588,293 @@
     <col min="7" max="7" width="13.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="5" t="s">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="4" spans="1:7" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B4" s="21" t="s">
         <v>33</v>
       </c>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="8"/>
-    </row>
-    <row r="2" spans="1:7" ht="34.799999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="19"/>
-      <c r="B2" s="7" t="s">
+      <c r="C4" s="23"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="23"/>
+      <c r="F4" s="23"/>
+      <c r="G4" s="22"/>
+    </row>
+    <row r="5" spans="1:7" ht="34.799999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="29"/>
+      <c r="B5" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="C2" s="8"/>
-      <c r="D2" s="7" t="s">
+      <c r="C5" s="22"/>
+      <c r="D5" s="21" t="s">
         <v>35</v>
       </c>
-      <c r="E2" s="8"/>
-      <c r="F2" s="7" t="s">
+      <c r="E5" s="22"/>
+      <c r="F5" s="21" t="s">
         <v>36</v>
       </c>
-      <c r="G2" s="8"/>
-    </row>
-    <row r="3" spans="1:7" ht="56.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="6"/>
-      <c r="B3" s="18"/>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
-      <c r="G3" s="18"/>
-    </row>
-    <row r="4" spans="1:7" ht="54.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="4" t="s">
+      <c r="G5" s="22"/>
+    </row>
+    <row r="6" spans="1:7" ht="56.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="20"/>
+      <c r="B6" s="12"/>
+      <c r="C6" s="12"/>
+      <c r="D6" s="12"/>
+      <c r="E6" s="12"/>
+      <c r="F6" s="12"/>
+      <c r="G6" s="12"/>
+    </row>
+    <row r="7" spans="1:7" ht="54.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B7" s="2">
         <v>1.36</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C7" s="2">
         <v>0.83</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D7" s="2">
         <v>1.27</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E7" s="2">
         <v>0.98</v>
       </c>
-      <c r="F4" s="2">
+      <c r="F7" s="2">
         <v>1.36</v>
       </c>
-      <c r="G4" s="2">
+      <c r="G7" s="2">
         <v>0.84</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="54.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="4" t="s">
+    <row r="8" spans="1:7" ht="54.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B8" s="2">
         <v>1.31</v>
       </c>
-      <c r="C5" s="2">
+      <c r="C8" s="2">
         <v>0.66</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D8" s="2">
         <v>1.24</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E8" s="2">
         <v>0.66</v>
       </c>
-      <c r="F5" s="2">
+      <c r="F8" s="2">
         <v>1.33</v>
       </c>
-      <c r="G5" s="2">
+      <c r="G8" s="2">
         <v>0.75</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="10" spans="1:7" ht="36.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="20" t="s">
+    <row r="12" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="13" spans="1:7" ht="36.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B13" s="21" t="s">
         <v>33</v>
       </c>
-      <c r="C10" s="9"/>
-      <c r="D10" s="9"/>
-      <c r="E10" s="9"/>
-      <c r="F10" s="9"/>
-      <c r="G10" s="8"/>
-    </row>
-    <row r="11" spans="1:7" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="21"/>
-      <c r="B11" s="7" t="s">
+      <c r="C13" s="23"/>
+      <c r="D13" s="23"/>
+      <c r="E13" s="23"/>
+      <c r="F13" s="23"/>
+      <c r="G13" s="22"/>
+    </row>
+    <row r="14" spans="1:7" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="14"/>
+      <c r="B14" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="C11" s="8"/>
-      <c r="D11" s="7" t="s">
+      <c r="C14" s="22"/>
+      <c r="D14" s="21" t="s">
         <v>35</v>
       </c>
-      <c r="E11" s="8"/>
-      <c r="F11" s="7" t="s">
+      <c r="E14" s="22"/>
+      <c r="F14" s="21" t="s">
         <v>36</v>
       </c>
-      <c r="G11" s="8"/>
-    </row>
-    <row r="12" spans="1:7" ht="54.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="4" t="s">
+      <c r="G14" s="22"/>
+    </row>
+    <row r="15" spans="1:7" ht="54.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="B12" s="2">
+      <c r="B15" s="2">
         <v>1.36</v>
       </c>
-      <c r="C12" s="2">
+      <c r="C15" s="2">
         <v>0.83</v>
       </c>
-      <c r="D12" s="2">
+      <c r="D15" s="2">
         <v>1.27</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E15" s="2">
         <v>0.98</v>
       </c>
-      <c r="F12" s="2">
+      <c r="F15" s="2">
         <v>1.36</v>
       </c>
-      <c r="G12" s="2">
+      <c r="G15" s="2">
         <v>0.84</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="54.6" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="4" t="s">
+    <row r="16" spans="1:7" ht="54.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="B13" s="2">
+      <c r="B16" s="2">
         <v>1.31</v>
       </c>
-      <c r="C13" s="2">
+      <c r="C16" s="2">
         <v>0.66</v>
       </c>
-      <c r="D13" s="2">
+      <c r="D16" s="2">
         <v>1.24</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E16" s="2">
         <v>0.66</v>
       </c>
-      <c r="F13" s="2">
+      <c r="F16" s="2">
         <v>1.33</v>
       </c>
-      <c r="G13" s="2">
+      <c r="G16" s="2">
         <v>0.75</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="18" x14ac:dyDescent="0.3">
-      <c r="A14" s="22"/>
-      <c r="B14" s="22"/>
-      <c r="C14" s="22"/>
-      <c r="D14" s="22"/>
-      <c r="E14" s="22"/>
-      <c r="F14" s="22"/>
-      <c r="G14" s="22"/>
-    </row>
-    <row r="15" spans="1:7" ht="18" x14ac:dyDescent="0.3">
-      <c r="A15" s="22"/>
-      <c r="B15" s="22"/>
-      <c r="C15" s="22"/>
-      <c r="D15" s="22"/>
-      <c r="E15" s="22"/>
-      <c r="F15" s="22"/>
-      <c r="G15" s="22"/>
-    </row>
-    <row r="16" spans="1:7" ht="18" x14ac:dyDescent="0.3">
-      <c r="A16" s="22"/>
-      <c r="B16" s="22"/>
-      <c r="C16" s="22"/>
-      <c r="D16" s="22"/>
-      <c r="E16" s="22"/>
-      <c r="F16" s="22"/>
-      <c r="G16" s="22"/>
-    </row>
     <row r="17" spans="1:7" ht="18" x14ac:dyDescent="0.3">
-      <c r="A17" s="22"/>
-      <c r="B17" s="22"/>
-      <c r="C17" s="22"/>
-      <c r="D17" s="22"/>
-      <c r="E17" s="22"/>
-      <c r="F17" s="22"/>
-      <c r="G17" s="22"/>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A18" s="23"/>
-      <c r="B18" s="23"/>
-      <c r="C18" s="24" t="s">
+      <c r="A17" s="15"/>
+      <c r="B17" s="15"/>
+      <c r="C17" s="15"/>
+      <c r="D17" s="15"/>
+      <c r="E17" s="15"/>
+      <c r="F17" s="15"/>
+      <c r="G17" s="15"/>
+    </row>
+    <row r="18" spans="1:7" ht="18" x14ac:dyDescent="0.3">
+      <c r="A18" s="15"/>
+      <c r="B18" s="15"/>
+      <c r="C18" s="15"/>
+      <c r="D18" s="15"/>
+      <c r="E18" s="15"/>
+      <c r="F18" s="15"/>
+      <c r="G18" s="15"/>
+    </row>
+    <row r="19" spans="1:7" ht="18" x14ac:dyDescent="0.3">
+      <c r="A19" s="15"/>
+      <c r="B19" s="15"/>
+      <c r="C19" s="15"/>
+      <c r="D19" s="15"/>
+      <c r="E19" s="15"/>
+      <c r="F19" s="15"/>
+      <c r="G19" s="15"/>
+    </row>
+    <row r="20" spans="1:7" ht="18" x14ac:dyDescent="0.3">
+      <c r="A20" s="15"/>
+      <c r="B20" s="15"/>
+      <c r="C20" s="15"/>
+      <c r="D20" s="15"/>
+      <c r="E20" s="15"/>
+      <c r="F20" s="15"/>
+      <c r="G20" s="15"/>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A21" s="16"/>
+      <c r="B21" s="16"/>
+      <c r="C21" s="28" t="s">
         <v>39</v>
       </c>
-      <c r="D18" s="24"/>
-      <c r="E18" s="25" t="s">
+      <c r="D21" s="28"/>
+      <c r="E21" s="27" t="s">
         <v>40</v>
       </c>
-      <c r="F18" s="25"/>
-    </row>
-    <row r="19" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="27" t="s">
+      <c r="F21" s="27"/>
+    </row>
+    <row r="22" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="B19" s="27" t="s">
+      <c r="B22" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="C19" s="26">
+      <c r="C22" s="17">
         <v>1.36</v>
       </c>
-      <c r="D19" s="26">
+      <c r="D22" s="17">
         <v>0.83</v>
       </c>
-      <c r="E19" s="26">
+      <c r="E22" s="17">
         <v>1.31</v>
       </c>
-      <c r="F19" s="26">
+      <c r="F22" s="17">
         <v>0.66</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="27" t="s">
+    <row r="23" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="B20" s="27" t="s">
+      <c r="B23" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="C20" s="26">
+      <c r="C23" s="17">
         <v>1.27</v>
       </c>
-      <c r="D20" s="26">
+      <c r="D23" s="17">
         <v>0.98</v>
       </c>
-      <c r="E20" s="26">
+      <c r="E23" s="17">
         <v>1.24</v>
       </c>
-      <c r="F20" s="26">
+      <c r="F23" s="17">
         <v>0.66</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="27" t="s">
+    <row r="24" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="B21" s="27" t="s">
+      <c r="B24" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="C21" s="26">
+      <c r="C24" s="17">
         <v>1.36</v>
       </c>
-      <c r="D21" s="26">
+      <c r="D24" s="17">
         <v>0.84</v>
       </c>
-      <c r="E21" s="26">
+      <c r="E24" s="17">
         <v>1.33</v>
       </c>
-      <c r="F21" s="26">
+      <c r="F24" s="17">
         <v>0.75</v>
       </c>
     </row>
-    <row r="35" ht="36" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="36" ht="64.2" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="38" ht="36" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="39" ht="64.2" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="E18:F18"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="A1:A3"/>
-    <mergeCell ref="B1:G1"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="B10:G10"/>
+    <mergeCell ref="B13:G13"/>
+    <mergeCell ref="A4:A6"/>
+    <mergeCell ref="B4:G4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="E21:F21"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="F14:G14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3057,13 +4888,13 @@
               <from>
                 <xdr:col>1</xdr:col>
                 <xdr:colOff>0</xdr:colOff>
-                <xdr:row>2</xdr:row>
+                <xdr:row>5</xdr:row>
                 <xdr:rowOff>0</xdr:rowOff>
               </from>
               <to>
                 <xdr:col>2</xdr:col>
                 <xdr:colOff>0</xdr:colOff>
-                <xdr:row>2</xdr:row>
+                <xdr:row>5</xdr:row>
                 <xdr:rowOff>617220</xdr:rowOff>
               </to>
             </anchor>
@@ -3082,13 +4913,13 @@
               <from>
                 <xdr:col>2</xdr:col>
                 <xdr:colOff>106680</xdr:colOff>
-                <xdr:row>2</xdr:row>
+                <xdr:row>5</xdr:row>
                 <xdr:rowOff>53340</xdr:rowOff>
               </from>
               <to>
                 <xdr:col>2</xdr:col>
                 <xdr:colOff>1074420</xdr:colOff>
-                <xdr:row>2</xdr:row>
+                <xdr:row>5</xdr:row>
                 <xdr:rowOff>731520</xdr:rowOff>
               </to>
             </anchor>
@@ -3107,13 +4938,13 @@
               <from>
                 <xdr:col>3</xdr:col>
                 <xdr:colOff>0</xdr:colOff>
-                <xdr:row>2</xdr:row>
+                <xdr:row>5</xdr:row>
                 <xdr:rowOff>0</xdr:rowOff>
               </from>
               <to>
                 <xdr:col>3</xdr:col>
                 <xdr:colOff>1135380</xdr:colOff>
-                <xdr:row>2</xdr:row>
+                <xdr:row>5</xdr:row>
                 <xdr:rowOff>670560</xdr:rowOff>
               </to>
             </anchor>
@@ -3132,13 +4963,13 @@
               <from>
                 <xdr:col>4</xdr:col>
                 <xdr:colOff>0</xdr:colOff>
-                <xdr:row>2</xdr:row>
+                <xdr:row>5</xdr:row>
                 <xdr:rowOff>0</xdr:rowOff>
               </from>
               <to>
                 <xdr:col>4</xdr:col>
                 <xdr:colOff>944880</xdr:colOff>
-                <xdr:row>2</xdr:row>
+                <xdr:row>5</xdr:row>
                 <xdr:rowOff>731520</xdr:rowOff>
               </to>
             </anchor>
@@ -3157,13 +4988,13 @@
               <from>
                 <xdr:col>5</xdr:col>
                 <xdr:colOff>0</xdr:colOff>
-                <xdr:row>2</xdr:row>
+                <xdr:row>5</xdr:row>
                 <xdr:rowOff>0</xdr:rowOff>
               </from>
               <to>
                 <xdr:col>5</xdr:col>
                 <xdr:colOff>1013460</xdr:colOff>
-                <xdr:row>2</xdr:row>
+                <xdr:row>5</xdr:row>
                 <xdr:rowOff>678180</xdr:rowOff>
               </to>
             </anchor>
@@ -3182,13 +5013,13 @@
               <from>
                 <xdr:col>6</xdr:col>
                 <xdr:colOff>0</xdr:colOff>
-                <xdr:row>2</xdr:row>
+                <xdr:row>5</xdr:row>
                 <xdr:rowOff>0</xdr:rowOff>
               </from>
               <to>
                 <xdr:col>6</xdr:col>
                 <xdr:colOff>868680</xdr:colOff>
-                <xdr:row>2</xdr:row>
+                <xdr:row>5</xdr:row>
                 <xdr:rowOff>754380</xdr:rowOff>
               </to>
             </anchor>
@@ -3205,9 +5036,1433 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+  <dimension ref="B3:M11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <cols>
+    <col min="2" max="2" width="11.109375" customWidth="1"/>
+    <col min="13" max="13" width="4.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="F3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="4" spans="2:13" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B4" s="31"/>
+    </row>
+    <row r="5" spans="2:13" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B5" s="19" t="s">
+        <v>46</v>
+      </c>
+      <c r="C5" s="21" t="s">
+        <v>47</v>
+      </c>
+      <c r="D5" s="23"/>
+      <c r="E5" s="23"/>
+      <c r="F5" s="23"/>
+      <c r="G5" s="23"/>
+      <c r="H5" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="I5" s="23"/>
+      <c r="J5" s="23"/>
+      <c r="K5" s="23"/>
+      <c r="L5" s="47"/>
+      <c r="M5" s="41"/>
+    </row>
+    <row r="6" spans="2:13" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B6" s="29"/>
+      <c r="C6" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="D6" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="E6" s="23"/>
+      <c r="F6" s="23"/>
+      <c r="G6" s="23"/>
+      <c r="H6" s="45" t="s">
+        <v>5</v>
+      </c>
+      <c r="I6" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="J6" s="23"/>
+      <c r="K6" s="23"/>
+      <c r="L6" s="47"/>
+      <c r="M6" s="42"/>
+    </row>
+    <row r="7" spans="2:13" ht="54" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B7" s="20"/>
+      <c r="C7" s="26"/>
+      <c r="D7" s="32" t="s">
+        <v>50</v>
+      </c>
+      <c r="E7" s="32" t="s">
+        <v>51</v>
+      </c>
+      <c r="F7" s="32" t="s">
+        <v>52</v>
+      </c>
+      <c r="G7" s="43" t="s">
+        <v>53</v>
+      </c>
+      <c r="H7" s="46"/>
+      <c r="I7" s="44" t="s">
+        <v>50</v>
+      </c>
+      <c r="J7" s="44" t="s">
+        <v>51</v>
+      </c>
+      <c r="K7" s="44" t="s">
+        <v>52</v>
+      </c>
+      <c r="L7" s="44" t="s">
+        <v>53</v>
+      </c>
+      <c r="M7" s="33"/>
+    </row>
+    <row r="8" spans="2:13" ht="35.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B8" s="40" t="s">
+        <v>54</v>
+      </c>
+      <c r="C8" s="2">
+        <v>26</v>
+      </c>
+      <c r="D8" s="2">
+        <v>4</v>
+      </c>
+      <c r="E8" s="2">
+        <v>12</v>
+      </c>
+      <c r="F8" s="2">
+        <v>6</v>
+      </c>
+      <c r="G8" s="2">
+        <v>6</v>
+      </c>
+      <c r="H8" s="2">
+        <v>28</v>
+      </c>
+      <c r="I8" s="2">
+        <v>3</v>
+      </c>
+      <c r="J8" s="2">
+        <v>11</v>
+      </c>
+      <c r="K8" s="2">
+        <v>12</v>
+      </c>
+      <c r="L8" s="35"/>
+      <c r="M8" s="33"/>
+    </row>
+    <row r="9" spans="2:13" ht="35.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B9" s="40" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" s="2">
+        <v>25</v>
+      </c>
+      <c r="D9" s="2">
+        <v>3</v>
+      </c>
+      <c r="E9" s="2">
+        <v>10</v>
+      </c>
+      <c r="F9" s="2">
+        <v>8</v>
+      </c>
+      <c r="G9" s="2">
+        <v>4</v>
+      </c>
+      <c r="H9" s="2">
+        <v>26</v>
+      </c>
+      <c r="I9" s="2">
+        <v>2</v>
+      </c>
+      <c r="J9" s="2">
+        <v>11</v>
+      </c>
+      <c r="K9" s="2">
+        <v>13</v>
+      </c>
+      <c r="L9" s="35"/>
+      <c r="M9" s="33"/>
+    </row>
+    <row r="10" spans="2:13" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B10" s="34"/>
+      <c r="C10" s="2">
+        <f>C8+C9</f>
+        <v>51</v>
+      </c>
+      <c r="D10" s="2">
+        <f t="shared" ref="D10:L10" si="0">D8+D9</f>
+        <v>7</v>
+      </c>
+      <c r="E10" s="2">
+        <f t="shared" si="0"/>
+        <v>22</v>
+      </c>
+      <c r="F10" s="2">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="G10" s="2">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="H10" s="2">
+        <f t="shared" si="0"/>
+        <v>54</v>
+      </c>
+      <c r="I10" s="2">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="J10" s="2">
+        <f t="shared" si="0"/>
+        <v>22</v>
+      </c>
+      <c r="K10" s="2">
+        <f t="shared" si="0"/>
+        <v>25</v>
+      </c>
+      <c r="L10" s="2"/>
+      <c r="M10" s="33"/>
+    </row>
+    <row r="11" spans="2:13" ht="18" x14ac:dyDescent="0.3">
+      <c r="B11" s="39"/>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="B5:B7"/>
+    <mergeCell ref="C5:G5"/>
+    <mergeCell ref="C6:C7"/>
+    <mergeCell ref="D6:G6"/>
+    <mergeCell ref="H6:H7"/>
+    <mergeCell ref="I6:L6"/>
+    <mergeCell ref="H5:L5"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="B4:L12"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="4" spans="2:12" ht="18" x14ac:dyDescent="0.35">
+      <c r="C4" s="48" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="6" spans="2:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="7" spans="2:12" ht="31.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B7" s="19" t="s">
+        <v>46</v>
+      </c>
+      <c r="C7" s="21" t="s">
+        <v>47</v>
+      </c>
+      <c r="D7" s="23"/>
+      <c r="E7" s="23"/>
+      <c r="F7" s="23"/>
+      <c r="G7" s="22"/>
+      <c r="H7" s="37" t="s">
+        <v>48</v>
+      </c>
+      <c r="I7" s="36"/>
+      <c r="J7" s="36"/>
+      <c r="K7" s="36"/>
+      <c r="L7" s="38"/>
+    </row>
+    <row r="8" spans="2:12" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B8" s="29"/>
+      <c r="C8" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="D8" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="E8" s="23"/>
+      <c r="F8" s="23"/>
+      <c r="G8" s="22"/>
+      <c r="H8" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="I8" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="J8" s="23"/>
+      <c r="K8" s="23"/>
+      <c r="L8" s="22"/>
+    </row>
+    <row r="9" spans="2:12" ht="58.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B9" s="20"/>
+      <c r="C9" s="26"/>
+      <c r="D9" s="32" t="s">
+        <v>50</v>
+      </c>
+      <c r="E9" s="32" t="s">
+        <v>51</v>
+      </c>
+      <c r="F9" s="32" t="s">
+        <v>52</v>
+      </c>
+      <c r="G9" s="32" t="s">
+        <v>53</v>
+      </c>
+      <c r="H9" s="26"/>
+      <c r="I9" s="32" t="s">
+        <v>50</v>
+      </c>
+      <c r="J9" s="32" t="s">
+        <v>51</v>
+      </c>
+      <c r="K9" s="32" t="s">
+        <v>52</v>
+      </c>
+      <c r="L9" s="32" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="10" spans="2:12" ht="35.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B10" s="40" t="s">
+        <v>54</v>
+      </c>
+      <c r="C10" s="2">
+        <v>26</v>
+      </c>
+      <c r="D10" s="2">
+        <v>4</v>
+      </c>
+      <c r="E10" s="2">
+        <v>12</v>
+      </c>
+      <c r="F10" s="2">
+        <v>6</v>
+      </c>
+      <c r="G10" s="2">
+        <v>6</v>
+      </c>
+      <c r="H10" s="2">
+        <v>28</v>
+      </c>
+      <c r="I10" s="2">
+        <v>3</v>
+      </c>
+      <c r="J10" s="2">
+        <v>11</v>
+      </c>
+      <c r="K10" s="2">
+        <v>12</v>
+      </c>
+      <c r="L10" s="2"/>
+    </row>
+    <row r="11" spans="2:12" ht="35.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B11" s="40" t="s">
+        <v>8</v>
+      </c>
+      <c r="C11" s="2">
+        <v>25</v>
+      </c>
+      <c r="D11" s="2">
+        <v>3</v>
+      </c>
+      <c r="E11" s="2">
+        <v>10</v>
+      </c>
+      <c r="F11" s="2">
+        <v>8</v>
+      </c>
+      <c r="G11" s="2">
+        <v>4</v>
+      </c>
+      <c r="H11" s="2">
+        <v>26</v>
+      </c>
+      <c r="I11" s="2">
+        <v>2</v>
+      </c>
+      <c r="J11" s="2">
+        <v>11</v>
+      </c>
+      <c r="K11" s="2">
+        <v>13</v>
+      </c>
+      <c r="L11" s="2"/>
+    </row>
+    <row r="12" spans="2:12" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B12" s="40"/>
+      <c r="C12" s="2">
+        <f>C10+C11</f>
+        <v>51</v>
+      </c>
+      <c r="D12" s="2">
+        <f t="shared" ref="D12:L12" si="0">D10+D11</f>
+        <v>7</v>
+      </c>
+      <c r="E12" s="2">
+        <f t="shared" si="0"/>
+        <v>22</v>
+      </c>
+      <c r="F12" s="2">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="G12" s="2">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="H12" s="2">
+        <f t="shared" si="0"/>
+        <v>54</v>
+      </c>
+      <c r="I12" s="2">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="J12" s="2">
+        <f t="shared" si="0"/>
+        <v>22</v>
+      </c>
+      <c r="K12" s="2">
+        <f t="shared" si="0"/>
+        <v>25</v>
+      </c>
+      <c r="L12" s="2"/>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="B7:B9"/>
+    <mergeCell ref="C7:G7"/>
+    <mergeCell ref="H7:L7"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="D8:G8"/>
+    <mergeCell ref="H8:H9"/>
+    <mergeCell ref="I8:L8"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="C2:M9"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="2" spans="3:13" ht="18" x14ac:dyDescent="0.35">
+      <c r="D2" s="48" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="3" spans="3:13" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="4" spans="3:13" ht="28.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C4" s="19" t="s">
+        <v>46</v>
+      </c>
+      <c r="D4" s="21" t="s">
+        <v>47</v>
+      </c>
+      <c r="E4" s="23"/>
+      <c r="F4" s="23"/>
+      <c r="G4" s="23"/>
+      <c r="H4" s="22"/>
+      <c r="I4" s="37" t="s">
+        <v>48</v>
+      </c>
+      <c r="J4" s="36"/>
+      <c r="K4" s="36"/>
+      <c r="L4" s="36"/>
+      <c r="M4" s="38"/>
+    </row>
+    <row r="5" spans="3:13" ht="25.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C5" s="29"/>
+      <c r="D5" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="E5" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="F5" s="23"/>
+      <c r="G5" s="23"/>
+      <c r="H5" s="22"/>
+      <c r="I5" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="J5" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="K5" s="23"/>
+      <c r="L5" s="23"/>
+      <c r="M5" s="22"/>
+    </row>
+    <row r="6" spans="3:13" ht="53.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C6" s="20"/>
+      <c r="D6" s="26"/>
+      <c r="E6" s="32" t="s">
+        <v>50</v>
+      </c>
+      <c r="F6" s="32" t="s">
+        <v>51</v>
+      </c>
+      <c r="G6" s="32" t="s">
+        <v>52</v>
+      </c>
+      <c r="H6" s="32" t="s">
+        <v>53</v>
+      </c>
+      <c r="I6" s="26"/>
+      <c r="J6" s="32" t="s">
+        <v>50</v>
+      </c>
+      <c r="K6" s="32" t="s">
+        <v>51</v>
+      </c>
+      <c r="L6" s="32" t="s">
+        <v>52</v>
+      </c>
+      <c r="M6" s="32" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="7" spans="3:13" ht="35.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C7" s="40" t="s">
+        <v>54</v>
+      </c>
+      <c r="D7" s="2">
+        <v>26</v>
+      </c>
+      <c r="E7" s="2">
+        <v>4</v>
+      </c>
+      <c r="F7" s="2">
+        <v>12</v>
+      </c>
+      <c r="G7" s="2">
+        <v>6</v>
+      </c>
+      <c r="H7" s="2">
+        <v>6</v>
+      </c>
+      <c r="I7" s="2">
+        <v>28</v>
+      </c>
+      <c r="J7" s="2">
+        <v>3</v>
+      </c>
+      <c r="K7" s="2">
+        <v>11</v>
+      </c>
+      <c r="L7" s="2">
+        <v>12</v>
+      </c>
+      <c r="M7" s="2"/>
+    </row>
+    <row r="8" spans="3:13" ht="35.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C8" s="40" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" s="2">
+        <v>25</v>
+      </c>
+      <c r="E8" s="2">
+        <v>3</v>
+      </c>
+      <c r="F8" s="2">
+        <v>10</v>
+      </c>
+      <c r="G8" s="2">
+        <v>8</v>
+      </c>
+      <c r="H8" s="2">
+        <v>4</v>
+      </c>
+      <c r="I8" s="2">
+        <v>26</v>
+      </c>
+      <c r="J8" s="2">
+        <v>2</v>
+      </c>
+      <c r="K8" s="2">
+        <v>11</v>
+      </c>
+      <c r="L8" s="2">
+        <v>13</v>
+      </c>
+      <c r="M8" s="2"/>
+    </row>
+    <row r="9" spans="3:13" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C9" s="40"/>
+      <c r="D9" s="2">
+        <f>D7+D8</f>
+        <v>51</v>
+      </c>
+      <c r="E9" s="2">
+        <f t="shared" ref="E9:M9" si="0">E7+E8</f>
+        <v>7</v>
+      </c>
+      <c r="F9" s="2">
+        <f t="shared" si="0"/>
+        <v>22</v>
+      </c>
+      <c r="G9" s="2">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="H9" s="2">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="I9" s="2">
+        <f t="shared" si="0"/>
+        <v>54</v>
+      </c>
+      <c r="J9" s="2">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="K9" s="2">
+        <f t="shared" si="0"/>
+        <v>22</v>
+      </c>
+      <c r="L9" s="2">
+        <f t="shared" si="0"/>
+        <v>25</v>
+      </c>
+      <c r="M9" s="2"/>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="C4:C6"/>
+    <mergeCell ref="D4:H4"/>
+    <mergeCell ref="I4:M4"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:H5"/>
+    <mergeCell ref="I5:I6"/>
+    <mergeCell ref="J5:M5"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="C2:H6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="3" max="3" width="16.88671875" customWidth="1"/>
+    <col min="4" max="4" width="17.77734375" customWidth="1"/>
+    <col min="5" max="6" width="17.21875" customWidth="1"/>
+    <col min="7" max="7" width="18.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="3:8" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C2" s="39" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="3" spans="3:8" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C3" s="49" t="s">
+        <v>58</v>
+      </c>
+      <c r="D3" s="50" t="s">
+        <v>50</v>
+      </c>
+      <c r="E3" s="50" t="s">
+        <v>51</v>
+      </c>
+      <c r="F3" s="50" t="s">
+        <v>52</v>
+      </c>
+      <c r="G3" s="50" t="s">
+        <v>53</v>
+      </c>
+      <c r="H3" s="50"/>
+    </row>
+    <row r="4" spans="3:8" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C4" s="51" t="s">
+        <v>47</v>
+      </c>
+      <c r="D4" s="52"/>
+      <c r="E4" s="52"/>
+      <c r="F4" s="52"/>
+      <c r="G4" s="52"/>
+      <c r="H4" s="52"/>
+    </row>
+    <row r="5" spans="3:8" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C5" s="51" t="s">
+        <v>59</v>
+      </c>
+      <c r="D5" s="52"/>
+      <c r="E5" s="52"/>
+      <c r="F5" s="52"/>
+      <c r="G5" s="52"/>
+      <c r="H5" s="52"/>
+    </row>
+    <row r="6" spans="3:8" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C6" s="51"/>
+      <c r="D6" s="52"/>
+      <c r="E6" s="52"/>
+      <c r="F6" s="52"/>
+      <c r="G6" s="52"/>
+      <c r="H6" s="35"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
+  <oleObjects>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice Requires="x14">
+        <oleObject progId="Equation.3" shapeId="11278" r:id="rId3">
+          <objectPr defaultSize="0" autoPict="0" r:id="rId4">
+            <anchor moveWithCells="1" sizeWithCells="1">
+              <from>
+                <xdr:col>3</xdr:col>
+                <xdr:colOff>0</xdr:colOff>
+                <xdr:row>3</xdr:row>
+                <xdr:rowOff>0</xdr:rowOff>
+              </from>
+              <to>
+                <xdr:col>3</xdr:col>
+                <xdr:colOff>487680</xdr:colOff>
+                <xdr:row>3</xdr:row>
+                <xdr:rowOff>220980</xdr:rowOff>
+              </to>
+            </anchor>
+          </objectPr>
+        </oleObject>
+      </mc:Choice>
+      <mc:Fallback>
+        <oleObject progId="Equation.3" shapeId="11278" r:id="rId3"/>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice Requires="x14">
+        <oleObject progId="Equation.3" shapeId="11277" r:id="rId5">
+          <objectPr defaultSize="0" autoPict="0" r:id="rId6">
+            <anchor moveWithCells="1" sizeWithCells="1">
+              <from>
+                <xdr:col>4</xdr:col>
+                <xdr:colOff>0</xdr:colOff>
+                <xdr:row>3</xdr:row>
+                <xdr:rowOff>0</xdr:rowOff>
+              </from>
+              <to>
+                <xdr:col>4</xdr:col>
+                <xdr:colOff>487680</xdr:colOff>
+                <xdr:row>3</xdr:row>
+                <xdr:rowOff>220980</xdr:rowOff>
+              </to>
+            </anchor>
+          </objectPr>
+        </oleObject>
+      </mc:Choice>
+      <mc:Fallback>
+        <oleObject progId="Equation.3" shapeId="11277" r:id="rId5"/>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice Requires="x14">
+        <oleObject progId="Equation.3" shapeId="11276" r:id="rId7">
+          <objectPr defaultSize="0" autoPict="0" r:id="rId8">
+            <anchor moveWithCells="1" sizeWithCells="1">
+              <from>
+                <xdr:col>5</xdr:col>
+                <xdr:colOff>0</xdr:colOff>
+                <xdr:row>3</xdr:row>
+                <xdr:rowOff>0</xdr:rowOff>
+              </from>
+              <to>
+                <xdr:col>5</xdr:col>
+                <xdr:colOff>541020</xdr:colOff>
+                <xdr:row>3</xdr:row>
+                <xdr:rowOff>228600</xdr:rowOff>
+              </to>
+            </anchor>
+          </objectPr>
+        </oleObject>
+      </mc:Choice>
+      <mc:Fallback>
+        <oleObject progId="Equation.3" shapeId="11276" r:id="rId7"/>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice Requires="x14">
+        <oleObject progId="Equation.3" shapeId="11275" r:id="rId9">
+          <objectPr defaultSize="0" autoPict="0" r:id="rId10">
+            <anchor moveWithCells="1" sizeWithCells="1">
+              <from>
+                <xdr:col>6</xdr:col>
+                <xdr:colOff>0</xdr:colOff>
+                <xdr:row>3</xdr:row>
+                <xdr:rowOff>0</xdr:rowOff>
+              </from>
+              <to>
+                <xdr:col>6</xdr:col>
+                <xdr:colOff>495300</xdr:colOff>
+                <xdr:row>3</xdr:row>
+                <xdr:rowOff>220980</xdr:rowOff>
+              </to>
+            </anchor>
+          </objectPr>
+        </oleObject>
+      </mc:Choice>
+      <mc:Fallback>
+        <oleObject progId="Equation.3" shapeId="11275" r:id="rId9"/>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice Requires="x14">
+        <oleObject progId="Equation.3" shapeId="11274" r:id="rId11">
+          <objectPr defaultSize="0" autoPict="0" r:id="rId12">
+            <anchor moveWithCells="1" sizeWithCells="1">
+              <from>
+                <xdr:col>7</xdr:col>
+                <xdr:colOff>0</xdr:colOff>
+                <xdr:row>3</xdr:row>
+                <xdr:rowOff>0</xdr:rowOff>
+              </from>
+              <to>
+                <xdr:col>7</xdr:col>
+                <xdr:colOff>480060</xdr:colOff>
+                <xdr:row>3</xdr:row>
+                <xdr:rowOff>220980</xdr:rowOff>
+              </to>
+            </anchor>
+          </objectPr>
+        </oleObject>
+      </mc:Choice>
+      <mc:Fallback>
+        <oleObject progId="Equation.3" shapeId="11274" r:id="rId11"/>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice Requires="x14">
+        <oleObject progId="Equation.3" shapeId="11273" r:id="rId13">
+          <objectPr defaultSize="0" autoPict="0" r:id="rId14">
+            <anchor moveWithCells="1" sizeWithCells="1">
+              <from>
+                <xdr:col>3</xdr:col>
+                <xdr:colOff>0</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>0</xdr:rowOff>
+              </from>
+              <to>
+                <xdr:col>3</xdr:col>
+                <xdr:colOff>480060</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>220980</xdr:rowOff>
+              </to>
+            </anchor>
+          </objectPr>
+        </oleObject>
+      </mc:Choice>
+      <mc:Fallback>
+        <oleObject progId="Equation.3" shapeId="11273" r:id="rId13"/>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice Requires="x14">
+        <oleObject progId="Equation.3" shapeId="11272" r:id="rId15">
+          <objectPr defaultSize="0" autoPict="0" r:id="rId16">
+            <anchor moveWithCells="1" sizeWithCells="1">
+              <from>
+                <xdr:col>4</xdr:col>
+                <xdr:colOff>0</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>0</xdr:rowOff>
+              </from>
+              <to>
+                <xdr:col>4</xdr:col>
+                <xdr:colOff>502920</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>220980</xdr:rowOff>
+              </to>
+            </anchor>
+          </objectPr>
+        </oleObject>
+      </mc:Choice>
+      <mc:Fallback>
+        <oleObject progId="Equation.3" shapeId="11272" r:id="rId15"/>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice Requires="x14">
+        <oleObject progId="Equation.3" shapeId="11271" r:id="rId17">
+          <objectPr defaultSize="0" autoPict="0" r:id="rId18">
+            <anchor moveWithCells="1" sizeWithCells="1">
+              <from>
+                <xdr:col>5</xdr:col>
+                <xdr:colOff>0</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>0</xdr:rowOff>
+              </from>
+              <to>
+                <xdr:col>5</xdr:col>
+                <xdr:colOff>563880</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>228600</xdr:rowOff>
+              </to>
+            </anchor>
+          </objectPr>
+        </oleObject>
+      </mc:Choice>
+      <mc:Fallback>
+        <oleObject progId="Equation.3" shapeId="11271" r:id="rId17"/>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice Requires="x14">
+        <oleObject progId="Equation.3" shapeId="11270" r:id="rId19">
+          <objectPr defaultSize="0" autoPict="0" r:id="rId20">
+            <anchor moveWithCells="1" sizeWithCells="1">
+              <from>
+                <xdr:col>6</xdr:col>
+                <xdr:colOff>0</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>0</xdr:rowOff>
+              </from>
+              <to>
+                <xdr:col>6</xdr:col>
+                <xdr:colOff>563880</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>220980</xdr:rowOff>
+              </to>
+            </anchor>
+          </objectPr>
+        </oleObject>
+      </mc:Choice>
+      <mc:Fallback>
+        <oleObject progId="Equation.3" shapeId="11270" r:id="rId19"/>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice Requires="x14">
+        <oleObject progId="Equation.3" shapeId="11269" r:id="rId21">
+          <objectPr defaultSize="0" autoPict="0" r:id="rId22">
+            <anchor moveWithCells="1" sizeWithCells="1">
+              <from>
+                <xdr:col>7</xdr:col>
+                <xdr:colOff>0</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>0</xdr:rowOff>
+              </from>
+              <to>
+                <xdr:col>7</xdr:col>
+                <xdr:colOff>487680</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>220980</xdr:rowOff>
+              </to>
+            </anchor>
+          </objectPr>
+        </oleObject>
+      </mc:Choice>
+      <mc:Fallback>
+        <oleObject progId="Equation.3" shapeId="11269" r:id="rId21"/>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice Requires="x14">
+        <oleObject progId="Equation.3" shapeId="11268" r:id="rId23">
+          <objectPr defaultSize="0" autoPict="0" r:id="rId24">
+            <anchor moveWithCells="1" sizeWithCells="1">
+              <from>
+                <xdr:col>3</xdr:col>
+                <xdr:colOff>0</xdr:colOff>
+                <xdr:row>5</xdr:row>
+                <xdr:rowOff>30480</xdr:rowOff>
+              </from>
+              <to>
+                <xdr:col>3</xdr:col>
+                <xdr:colOff>1196340</xdr:colOff>
+                <xdr:row>5</xdr:row>
+                <xdr:rowOff>213360</xdr:rowOff>
+              </to>
+            </anchor>
+          </objectPr>
+        </oleObject>
+      </mc:Choice>
+      <mc:Fallback>
+        <oleObject progId="Equation.3" shapeId="11268" r:id="rId23"/>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice Requires="x14">
+        <oleObject progId="Equation.3" shapeId="11267" r:id="rId25">
+          <objectPr defaultSize="0" autoPict="0" r:id="rId26">
+            <anchor moveWithCells="1" sizeWithCells="1">
+              <from>
+                <xdr:col>4</xdr:col>
+                <xdr:colOff>0</xdr:colOff>
+                <xdr:row>5</xdr:row>
+                <xdr:rowOff>53340</xdr:rowOff>
+              </from>
+              <to>
+                <xdr:col>4</xdr:col>
+                <xdr:colOff>1150620</xdr:colOff>
+                <xdr:row>5</xdr:row>
+                <xdr:rowOff>220980</xdr:rowOff>
+              </to>
+            </anchor>
+          </objectPr>
+        </oleObject>
+      </mc:Choice>
+      <mc:Fallback>
+        <oleObject progId="Equation.3" shapeId="11267" r:id="rId25"/>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice Requires="x14">
+        <oleObject progId="Equation.3" shapeId="11266" r:id="rId27">
+          <objectPr defaultSize="0" autoPict="0" r:id="rId28">
+            <anchor moveWithCells="1" sizeWithCells="1">
+              <from>
+                <xdr:col>5</xdr:col>
+                <xdr:colOff>0</xdr:colOff>
+                <xdr:row>5</xdr:row>
+                <xdr:rowOff>53340</xdr:rowOff>
+              </from>
+              <to>
+                <xdr:col>5</xdr:col>
+                <xdr:colOff>1158240</xdr:colOff>
+                <xdr:row>5</xdr:row>
+                <xdr:rowOff>228600</xdr:rowOff>
+              </to>
+            </anchor>
+          </objectPr>
+        </oleObject>
+      </mc:Choice>
+      <mc:Fallback>
+        <oleObject progId="Equation.3" shapeId="11266" r:id="rId27"/>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice Requires="x14">
+        <oleObject progId="Equation.3" shapeId="11265" r:id="rId29">
+          <objectPr defaultSize="0" autoPict="0" r:id="rId30">
+            <anchor moveWithCells="1" sizeWithCells="1">
+              <from>
+                <xdr:col>6</xdr:col>
+                <xdr:colOff>0</xdr:colOff>
+                <xdr:row>5</xdr:row>
+                <xdr:rowOff>45720</xdr:rowOff>
+              </from>
+              <to>
+                <xdr:col>6</xdr:col>
+                <xdr:colOff>1264920</xdr:colOff>
+                <xdr:row>5</xdr:row>
+                <xdr:rowOff>220980</xdr:rowOff>
+              </to>
+            </anchor>
+          </objectPr>
+        </oleObject>
+      </mc:Choice>
+      <mc:Fallback>
+        <oleObject progId="Equation.3" shapeId="11265" r:id="rId29"/>
+      </mc:Fallback>
+    </mc:AlternateContent>
+  </oleObjects>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="B2:O14"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="3" max="3" width="18.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:15" ht="18" x14ac:dyDescent="0.3">
+      <c r="B2" s="53" t="s">
+        <v>60</v>
+      </c>
+      <c r="C2" s="53"/>
+      <c r="D2" s="53"/>
+      <c r="E2" s="53"/>
+      <c r="F2" s="53"/>
+      <c r="G2" s="53"/>
+      <c r="H2" s="53"/>
+      <c r="I2" s="53"/>
+      <c r="J2" s="53"/>
+    </row>
+    <row r="3" spans="2:15" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="4" spans="2:15" ht="32.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C4" s="57" t="s">
+        <v>46</v>
+      </c>
+      <c r="D4" s="59" t="s">
+        <v>61</v>
+      </c>
+      <c r="E4" s="23"/>
+      <c r="F4" s="23"/>
+      <c r="G4" s="60"/>
+      <c r="H4" s="61" t="s">
+        <v>62</v>
+      </c>
+      <c r="I4" s="36"/>
+      <c r="J4" s="36"/>
+      <c r="K4" s="62"/>
+      <c r="L4" s="63" t="s">
+        <v>63</v>
+      </c>
+      <c r="M4" s="65" t="s">
+        <v>64</v>
+      </c>
+      <c r="N4" s="67" t="s">
+        <v>65</v>
+      </c>
+      <c r="O4" s="67" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="5" spans="2:15" ht="73.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C5" s="58"/>
+      <c r="D5" s="32" t="s">
+        <v>50</v>
+      </c>
+      <c r="E5" s="32" t="s">
+        <v>51</v>
+      </c>
+      <c r="F5" s="32" t="s">
+        <v>52</v>
+      </c>
+      <c r="G5" s="54" t="s">
+        <v>53</v>
+      </c>
+      <c r="H5" s="32" t="s">
+        <v>50</v>
+      </c>
+      <c r="I5" s="32" t="s">
+        <v>51</v>
+      </c>
+      <c r="J5" s="32" t="s">
+        <v>52</v>
+      </c>
+      <c r="K5" s="54" t="s">
+        <v>53</v>
+      </c>
+      <c r="L5" s="64"/>
+      <c r="M5" s="66"/>
+      <c r="N5" s="68"/>
+      <c r="O5" s="68"/>
+    </row>
+    <row r="6" spans="2:15" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C6" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="D6" s="23"/>
+      <c r="E6" s="23"/>
+      <c r="F6" s="23"/>
+      <c r="G6" s="23"/>
+      <c r="H6" s="23"/>
+      <c r="I6" s="23"/>
+      <c r="J6" s="23"/>
+      <c r="K6" s="23"/>
+      <c r="L6" s="23"/>
+      <c r="M6" s="23"/>
+      <c r="N6" s="23"/>
+      <c r="O6" s="22"/>
+    </row>
+    <row r="7" spans="2:15" ht="21" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C7" s="55" t="s">
+        <v>54</v>
+      </c>
+      <c r="D7" s="35">
+        <v>2</v>
+      </c>
+      <c r="E7" s="35">
+        <v>8</v>
+      </c>
+      <c r="F7" s="35">
+        <v>10</v>
+      </c>
+      <c r="G7" s="56">
+        <v>6</v>
+      </c>
+      <c r="H7" s="35">
+        <v>1</v>
+      </c>
+      <c r="I7" s="35">
+        <v>7</v>
+      </c>
+      <c r="J7" s="35">
+        <v>10</v>
+      </c>
+      <c r="K7" s="56">
+        <v>10</v>
+      </c>
+      <c r="L7" s="35">
+        <v>26</v>
+      </c>
+      <c r="M7" s="35">
+        <v>28</v>
+      </c>
+      <c r="N7" s="35">
+        <v>1.33</v>
+      </c>
+      <c r="O7" s="35" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="8" spans="2:15" ht="21" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C8" s="55" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" s="35">
+        <v>2</v>
+      </c>
+      <c r="E8" s="35">
+        <v>7</v>
+      </c>
+      <c r="F8" s="35">
+        <v>8</v>
+      </c>
+      <c r="G8" s="56">
+        <v>8</v>
+      </c>
+      <c r="H8" s="35">
+        <v>2</v>
+      </c>
+      <c r="I8" s="35">
+        <v>5</v>
+      </c>
+      <c r="J8" s="35">
+        <v>10</v>
+      </c>
+      <c r="K8" s="56">
+        <v>9</v>
+      </c>
+      <c r="L8" s="35">
+        <v>25</v>
+      </c>
+      <c r="M8" s="35">
+        <v>26</v>
+      </c>
+      <c r="N8" s="35">
+        <v>0.6</v>
+      </c>
+      <c r="O8" s="35" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="9" spans="2:15" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C9" s="21" t="s">
+        <v>9</v>
+      </c>
+      <c r="D9" s="23"/>
+      <c r="E9" s="23"/>
+      <c r="F9" s="23"/>
+      <c r="G9" s="23"/>
+      <c r="H9" s="23"/>
+      <c r="I9" s="23"/>
+      <c r="J9" s="23"/>
+      <c r="K9" s="23"/>
+      <c r="L9" s="23"/>
+      <c r="M9" s="23"/>
+      <c r="N9" s="23"/>
+      <c r="O9" s="22"/>
+    </row>
+    <row r="10" spans="2:15" ht="21" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C10" s="55" t="s">
+        <v>54</v>
+      </c>
+      <c r="D10" s="35">
+        <v>2</v>
+      </c>
+      <c r="E10" s="35">
+        <v>8</v>
+      </c>
+      <c r="F10" s="35">
+        <v>10</v>
+      </c>
+      <c r="G10" s="56">
+        <v>6</v>
+      </c>
+      <c r="H10" s="35">
+        <v>1</v>
+      </c>
+      <c r="I10" s="35">
+        <v>7</v>
+      </c>
+      <c r="J10" s="35">
+        <v>10</v>
+      </c>
+      <c r="K10" s="56">
+        <v>10</v>
+      </c>
+      <c r="L10" s="35">
+        <v>26</v>
+      </c>
+      <c r="M10" s="35">
+        <v>28</v>
+      </c>
+      <c r="N10" s="35">
+        <v>1.33</v>
+      </c>
+      <c r="O10" s="35" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="11" spans="2:15" ht="21" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C11" s="55" t="s">
+        <v>8</v>
+      </c>
+      <c r="D11" s="35">
+        <v>2</v>
+      </c>
+      <c r="E11" s="35">
+        <v>7</v>
+      </c>
+      <c r="F11" s="35">
+        <v>8</v>
+      </c>
+      <c r="G11" s="56">
+        <v>8</v>
+      </c>
+      <c r="H11" s="35">
+        <v>2</v>
+      </c>
+      <c r="I11" s="35">
+        <v>5</v>
+      </c>
+      <c r="J11" s="35">
+        <v>10</v>
+      </c>
+      <c r="K11" s="56">
+        <v>9</v>
+      </c>
+      <c r="L11" s="35">
+        <v>25</v>
+      </c>
+      <c r="M11" s="35">
+        <v>26</v>
+      </c>
+      <c r="N11" s="35">
+        <v>0.6</v>
+      </c>
+      <c r="O11" s="35" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="12" spans="2:15" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C12" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="D12" s="23"/>
+      <c r="E12" s="23"/>
+      <c r="F12" s="23"/>
+      <c r="G12" s="23"/>
+      <c r="H12" s="23"/>
+      <c r="I12" s="23"/>
+      <c r="J12" s="23"/>
+      <c r="K12" s="23"/>
+      <c r="L12" s="23"/>
+      <c r="M12" s="23"/>
+      <c r="N12" s="23"/>
+      <c r="O12" s="22"/>
+    </row>
+    <row r="13" spans="2:15" ht="21" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C13" s="55" t="s">
+        <v>54</v>
+      </c>
+      <c r="D13" s="35">
+        <v>2</v>
+      </c>
+      <c r="E13" s="35">
+        <v>8</v>
+      </c>
+      <c r="F13" s="35">
+        <v>10</v>
+      </c>
+      <c r="G13" s="56">
+        <v>6</v>
+      </c>
+      <c r="H13" s="35">
+        <v>1</v>
+      </c>
+      <c r="I13" s="35">
+        <v>7</v>
+      </c>
+      <c r="J13" s="35">
+        <v>10</v>
+      </c>
+      <c r="K13" s="56">
+        <v>10</v>
+      </c>
+      <c r="L13" s="35">
+        <v>26</v>
+      </c>
+      <c r="M13" s="35">
+        <v>28</v>
+      </c>
+      <c r="N13" s="35">
+        <v>1.33</v>
+      </c>
+      <c r="O13" s="35" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="14" spans="2:15" ht="21" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C14" s="55" t="s">
+        <v>8</v>
+      </c>
+      <c r="D14" s="35">
+        <v>2</v>
+      </c>
+      <c r="E14" s="35">
+        <v>7</v>
+      </c>
+      <c r="F14" s="35">
+        <v>8</v>
+      </c>
+      <c r="G14" s="56">
+        <v>8</v>
+      </c>
+      <c r="H14" s="35">
+        <v>2</v>
+      </c>
+      <c r="I14" s="35">
+        <v>5</v>
+      </c>
+      <c r="J14" s="35">
+        <v>10</v>
+      </c>
+      <c r="K14" s="56">
+        <v>9</v>
+      </c>
+      <c r="L14" s="35">
+        <v>25</v>
+      </c>
+      <c r="M14" s="35">
+        <v>26</v>
+      </c>
+      <c r="N14" s="35">
+        <v>0.6</v>
+      </c>
+      <c r="O14" s="35" t="s">
+        <v>69</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="M4:M5"/>
+    <mergeCell ref="N4:N5"/>
+    <mergeCell ref="O4:O5"/>
+    <mergeCell ref="C6:O6"/>
+    <mergeCell ref="C9:O9"/>
+    <mergeCell ref="C12:O12"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="D4:G4"/>
+    <mergeCell ref="H4:K4"/>
+    <mergeCell ref="L4:L5"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>